<commit_message>
Publish EVT-PRE-20 REV_D8 with 21 and 41 procurement variants
</commit_message>
<xml_diff>
--- a/manufacturing/MFG_004_DIO_EVT_B01_EOL_MEASUREMENT_REGISTER_REV_A.xlsx
+++ b/manufacturing/MFG_004_DIO_EVT_B01_EOL_MEASUREMENT_REGISTER_REV_A.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R609e29ccbd954b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="2" r:id="R9544400e9d4f4aeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="3" r:id="Rdebc3da565be4e1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSA" sheetId="4" r:id="Rf76998916bd74090"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="5" r:id="R89a8bfd805634b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9b7d54b8439f4b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="2" r:id="Rd1ade1d5a11445c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="3" r:id="Rd9406f84a60b4ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSA" sheetId="4" r:id="R2cacbae5d3e1496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="5" r:id="R9546fb1f588448eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1307,7 +1307,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="14" t="str">
-        <x:v>OPEN limits</x:v>
+        <x:v>Открытые критерии / OPEN criteria (не число станций / not station count)</x:v>
       </x:c>
       <x:c r="B20" s="15" t="n">
         <x:v>21</x:v>
@@ -11013,7 +11013,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70fc3431c9ea4a76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7481a8c29bde46c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16890,7 +16890,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b5fc21d3594332"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R055142f581d24720"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21652,7 +21652,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd08e03f6f8d416c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf161787dc5514a55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26409,7 +26409,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Read69f9474fe48f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd39c36c41a8d448c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>